<commit_message>
adjust legends and colours
</commit_message>
<xml_diff>
--- a/appdata/threshold_definitions_delta_de.xlsx
+++ b/appdata/threshold_definitions_delta_de.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zhaw-my.sharepoint.com/personal/hedd_zhaw_ch/Documents/Dashboard Squarefoot Projekt/Squarefoot/Squarefoot code/squarefoot/appdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:9_{36C0AF89-E858-44E3-B955-074CA1A8DB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBA4CFBE-5BCA-47C2-BB44-524F1859E370}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:9_{36C0AF89-E858-44E3-B955-074CA1A8DB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DF4474D-6F50-49CB-BA07-4BE557F6005B}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{DF7BF7E8-8078-438A-9C9E-DC555A1DD317}"/>
+    <workbookView xWindow="-23148" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DF7BF7E8-8078-438A-9C9E-DC555A1DD317}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="2" r:id="rId1"/>
@@ -817,6 +817,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -1135,39 +1139,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E6735C-B05B-47AA-B7A1-6FD9EE6B912D}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>45684</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>33</v>
       </c>
@@ -1180,13 +1184,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{974DB341-E177-4541-8F5D-113D73DB9624}">
   <dimension ref="A1:P343"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.6640625" customWidth="1"/>
-    <col min="2" max="16" width="11.5546875" style="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="16" width="11.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1236,7 +1240,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1286,7 +1290,7 @@
         <v>-1.2254115E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1336,7 +1340,7 @@
         <v>6.7936407499999902E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1386,7 +1390,7 @@
         <v>4.0980859250000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1436,7 +1440,7 @@
         <v>1.385711825E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1486,7 +1490,7 @@
         <v>2.628505125E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1536,7 +1540,7 @@
         <v>1.294258E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1586,7 +1590,7 @@
         <v>1.24635625E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1636,7 +1640,7 @@
         <v>2.4525364000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1686,7 +1690,7 @@
         <v>-2.1170645249999901E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1736,7 +1740,7 @@
         <v>-1.4126566499999899E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1786,7 +1790,7 @@
         <v>-1.6168010499999899E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1836,7 +1840,7 @@
         <v>2.8080419999999902E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1886,7 +1890,7 @@
         <v>2.6755519999999999E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1936,7 +1940,7 @@
         <v>-6.7444069999999896E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1986,7 +1990,7 @@
         <v>-3.6168279999999899E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2036,7 +2040,7 @@
         <v>1.111301525E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2086,7 +2090,7 @@
         <v>3.3998322499999997E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2136,7 +2140,7 @@
         <v>-1.6468717500000001E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2186,7 +2190,7 @@
         <v>-2.253403075E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2236,7 +2240,7 @@
         <v>-6.4556557499999999E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2286,7 +2290,7 @@
         <v>-1.6978768999999901E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2336,7 +2340,7 @@
         <v>3.3480774999999998E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2386,7 +2390,7 @@
         <v>-1.0390791249999899E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2436,7 +2440,7 @@
         <v>-1.0590943499999899E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2486,7 +2490,7 @@
         <v>-1.5902989999999999E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2536,7 +2540,7 @@
         <v>5.3529267499999901E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2586,7 +2590,7 @@
         <v>1.6187571750000001E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2636,7 +2640,7 @@
         <v>-6.4967269999999999E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2686,7 +2690,7 @@
         <v>1.7429522121212099E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2736,7 +2740,7 @@
         <v>-4.2368724242424303E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2786,7 +2790,7 @@
         <v>-1.92155018181818E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2836,7 +2840,7 @@
         <v>2.8681689090908999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2886,7 +2890,7 @@
         <v>3.67948415151515E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2936,7 +2940,7 @@
         <v>1.66332606060606E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2986,7 +2990,7 @@
         <v>5.0113181818181697E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3036,7 +3040,7 @@
         <v>-2.57647818181817E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3086,7 +3090,7 @@
         <v>1.3343177878787801E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3136,7 +3140,7 @@
         <v>9.4864151515151492E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3186,7 +3190,7 @@
         <v>-1.8285824242424201E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3236,7 +3240,7 @@
         <v>2.2077455151515098E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3286,7 +3290,7 @@
         <v>1.20746396296296E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3336,7 +3340,7 @@
         <v>1.56437355555555E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3386,7 +3390,7 @@
         <v>3.3125228518518499E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3436,7 +3440,7 @@
         <v>-5.7563807407407302E-3</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3486,7 +3490,7 @@
         <v>3.8590781481481402E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3536,7 +3540,7 @@
         <v>-3.9280543703703603E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3586,7 +3590,7 @@
         <v>-4.98419562962963E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3636,7 +3640,7 @@
         <v>-5.1631509999999999E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3686,7 +3690,7 @@
         <v>-1.3612890370370299E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3736,7 +3740,7 @@
         <v>-1.64938248148148E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3786,7 +3790,7 @@
         <v>1.85459707407407E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -3836,7 +3840,7 @@
         <v>-8.0531637037036894E-3</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3886,7 +3890,7 @@
         <v>-4.9931681481481397E-3</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3936,7 +3940,7 @@
         <v>-6.7099785185185104E-3</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3986,7 +3990,7 @@
         <v>-2.2367998148148101E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4036,7 +4040,7 @@
         <v>-6.0274981481481501E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4086,7 +4090,7 @@
         <v>-1.02127525925925E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4136,7 +4140,7 @@
         <v>-5.14209407407408E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4186,7 +4190,7 @@
         <v>-1.6309683703703701E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -4236,7 +4240,7 @@
         <v>9.8421111111111599E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -4286,7 +4290,7 @@
         <v>-1.37015392592592E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -4336,7 +4340,7 @@
         <v>1.00039488888888E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -4386,7 +4390,7 @@
         <v>-2.02671944444444E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -4436,7 +4440,7 @@
         <v>-1.8053835925925899E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -4486,7 +4490,7 @@
         <v>-6.6917529629629598E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -4536,7 +4540,7 @@
         <v>2.95267555555556E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -4586,7 +4590,7 @@
         <v>-7.3819481481481397E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -4636,7 +4640,7 @@
         <v>8.9039107407407492E-3</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -4686,7 +4690,7 @@
         <v>2.89058144444444E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -4736,7 +4740,7 @@
         <v>2.98226766666666E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -4786,7 +4790,7 @@
         <v>3.86038999999999E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -4836,7 +4840,7 @@
         <v>7.3382724999999597E-3</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -4886,7 +4890,7 @@
         <v>-2.179557E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -4936,7 +4940,7 @@
         <v>6.8683725000000199E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -4986,7 +4990,7 @@
         <v>-2.70393224999999E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -5036,7 +5040,7 @@
         <v>-5.5811852499999898E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -5086,7 +5090,7 @@
         <v>-0.124401924999999</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -5136,7 +5140,7 @@
         <v>-7.2447667499999896E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -5186,7 +5190,7 @@
         <v>-5.6252690322580604E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -5236,7 +5240,7 @@
         <v>-5.7014042857142797E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -5286,7 +5290,7 @@
         <v>-6.0438220952380897E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -5336,7 +5340,7 @@
         <v>-2.9743096666666601E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -5386,7 +5390,7 @@
         <v>-7.9930190476190394E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -5436,7 +5440,7 @@
         <v>-1.25774003999999E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -5486,7 +5490,7 @@
         <v>-1.9948974025973899E-4</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -5536,7 +5540,7 @@
         <v>-4.4017604761904701E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -5586,7 +5590,7 @@
         <v>-1.1304480952381E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -5636,7 +5640,7 @@
         <v>-3.2570241904761897E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -5686,7 +5690,7 @@
         <v>-3.6306171428571298E-3</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -5736,7 +5740,7 @@
         <v>-6.70354714285714E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -5786,7 +5790,7 @@
         <v>-2.2714166666666599E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -5836,7 +5840,7 @@
         <v>-2.8279673599999899E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -5886,7 +5890,7 @@
         <v>-1.0797510476190399E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -5936,7 +5940,7 @@
         <v>-7.3818585714285701E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -5986,7 +5990,7 @@
         <v>-1.66396047619047E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -6036,7 +6040,7 @@
         <v>1.02542142857142E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -6086,7 +6090,7 @@
         <v>-1.0797033043478199E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -6136,7 +6140,7 @@
         <v>-1.8651839130434701E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -6186,7 +6190,7 @@
         <v>-1.2567943913043399E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -6236,7 +6240,7 @@
         <v>-1.4287544347826E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -6286,7 +6290,7 @@
         <v>-2.48834226086956E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -6336,7 +6340,7 @@
         <v>-2.8579854782608601E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -6386,7 +6390,7 @@
         <v>-1.9131555217391301E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -6436,7 +6440,7 @@
         <v>-3.5458034347825997E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>105</v>
       </c>
@@ -6486,7 +6490,7 @@
         <v>5.8076695652174595E-4</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -6536,7 +6540,7 @@
         <v>-1.99487104347826E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -6586,7 +6590,7 @@
         <v>-3.1249785217391201E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -6636,7 +6640,7 @@
         <v>-4.9979909565217299E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -6686,7 +6690,7 @@
         <v>-6.6968329411764699E-3</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -6736,7 +6740,7 @@
         <v>-2.40784294117647E-3</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -6786,7 +6790,7 @@
         <v>9.7946761904763101E-4</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -6836,7 +6840,7 @@
         <v>-8.0143209523809607E-3</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -6886,7 +6890,7 @@
         <v>-6.2071485714285503E-3</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -6936,7 +6940,7 @@
         <v>-2.3594607142857101E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -6986,7 +6990,7 @@
         <v>-4.5337576190476198E-3</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>116</v>
       </c>
@@ -7036,7 +7040,7 @@
         <v>-7.49587952380953E-3</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>117</v>
       </c>
@@ -7086,7 +7090,7 @@
         <v>-2.0690052380952402E-3</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>118</v>
       </c>
@@ -7136,7 +7140,7 @@
         <v>-1.6197409523809299E-3</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>119</v>
       </c>
@@ -7186,7 +7190,7 @@
         <v>-7.7743628571428601E-3</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>120</v>
       </c>
@@ -7236,7 +7240,7 @@
         <v>-1.3824469047619E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>121</v>
       </c>
@@ -7286,7 +7290,7 @@
         <v>-3.1108861904762001E-3</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>122</v>
       </c>
@@ -7336,7 +7340,7 @@
         <v>-7.87914761904762E-3</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>123</v>
       </c>
@@ -7386,7 +7390,7 @@
         <v>-3.4403738095237901E-3</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>124</v>
       </c>
@@ -7436,7 +7440,7 @@
         <v>8.5820047619046698E-4</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>125</v>
       </c>
@@ -7486,7 +7490,7 @@
         <v>-1.77160619047618E-3</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>126</v>
       </c>
@@ -7536,7 +7540,7 @@
         <v>1.1613714285714301E-3</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>127</v>
       </c>
@@ -7586,7 +7590,7 @@
         <v>3.2923547368420999E-3</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>128</v>
       </c>
@@ -7636,7 +7640,7 @@
         <v>-9.6799510526315701E-3</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>129</v>
       </c>
@@ -7686,7 +7690,7 @@
         <v>2.70191684210527E-3</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>130</v>
       </c>
@@ -7736,7 +7740,7 @@
         <v>-4.9820842105263302E-3</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>131</v>
       </c>
@@ -7786,7 +7790,7 @@
         <v>-1.3527493157894701E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>132</v>
       </c>
@@ -7836,7 +7840,7 @@
         <v>5.0753842105263104E-3</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>133</v>
       </c>
@@ -7886,7 +7890,7 @@
         <v>-3.4103052631577398E-4</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>134</v>
       </c>
@@ -7936,7 +7940,7 @@
         <v>-3.13201589473684E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>135</v>
       </c>
@@ -7986,7 +7990,7 @@
         <v>-6.7336484210526199E-3</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>136</v>
       </c>
@@ -8036,7 +8040,7 @@
         <v>-5.2901775263157799E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>137</v>
       </c>
@@ -8086,7 +8090,7 @@
         <v>-1.8588343684210501E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>138</v>
       </c>
@@ -8136,7 +8140,7 @@
         <v>-4.1953336842105301E-3</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>139</v>
       </c>
@@ -8186,7 +8190,7 @@
         <v>-4.53776684210526E-3</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>140</v>
       </c>
@@ -8236,7 +8240,7 @@
         <v>-9.32662105263145E-4</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>141</v>
       </c>
@@ -8286,7 +8290,7 @@
         <v>-2.8824863157894602E-3</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>142</v>
       </c>
@@ -8336,7 +8340,7 @@
         <v>-5.8589578947367297E-4</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>143</v>
       </c>
@@ -8386,7 +8390,7 @@
         <v>-3.1945978947368401E-3</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>144</v>
       </c>
@@ -8436,7 +8440,7 @@
         <v>-8.3140257894736801E-3</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>145</v>
       </c>
@@ -8486,7 +8490,7 @@
         <v>-5.40252736842106E-3</v>
       </c>
     </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>146</v>
       </c>
@@ -8536,7 +8540,7 @@
         <v>-8.4636831578947403E-3</v>
       </c>
     </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>147</v>
       </c>
@@ -8586,7 +8590,7 @@
         <v>-6.8457705882352896E-3</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>148</v>
       </c>
@@ -8636,7 +8640,7 @@
         <v>7.7992413333333399E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>149</v>
       </c>
@@ -8686,7 +8690,7 @@
         <v>-0.12454680999999999</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>150</v>
       </c>
@@ -8736,7 +8740,7 @@
         <v>-2.05602799999999E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>151</v>
       </c>
@@ -8786,7 +8790,7 @@
         <v>0.106106966666666</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>152</v>
       </c>
@@ -8836,7 +8840,7 @@
         <v>-0.21105627333333299</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>153</v>
       </c>
@@ -8886,7 +8890,7 @@
         <v>-2.3963633333332602E-3</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>154</v>
       </c>
@@ -8936,7 +8940,7 @@
         <v>-4.1248686666666701E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>155</v>
       </c>
@@ -8986,7 +8990,7 @@
         <v>-0.14215387333333299</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>156</v>
       </c>
@@ -9036,7 +9040,7 @@
         <v>8.3738063333333196E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>157</v>
       </c>
@@ -9086,7 +9090,7 @@
         <v>6.54923999999999E-3</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>158</v>
       </c>
@@ -9136,7 +9140,7 @@
         <v>4.4165233599999999E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>159</v>
       </c>
@@ -9186,7 +9190,7 @@
         <v>3.0298814399999999E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>160</v>
       </c>
@@ -9236,7 +9240,7 @@
         <v>-7.6263800000000003E-3</v>
       </c>
     </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>161</v>
       </c>
@@ -9286,7 +9290,7 @@
         <v>1.3330655599999901E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>162</v>
       </c>
@@ -9336,7 +9340,7 @@
         <v>-6.8435415200000002E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>163</v>
       </c>
@@ -9386,7 +9390,7 @@
         <v>-6.3468842400000003E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>164</v>
       </c>
@@ -9436,7 +9440,7 @@
         <v>-5.2665028799999999E-2</v>
       </c>
     </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>165</v>
       </c>
@@ -9486,7 +9490,7 @@
         <v>-2.1646467199999998E-2</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>166</v>
       </c>
@@ -9536,7 +9540,7 @@
         <v>-1.6337103200000001E-2</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>167</v>
       </c>
@@ -9586,7 +9590,7 @@
         <v>5.1152608399999903E-2</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>168</v>
       </c>
@@ -9636,7 +9640,7 @@
         <v>-9.9410083999999892E-3</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>169</v>
       </c>
@@ -9686,7 +9690,7 @@
         <v>-9.5689828000000005E-3</v>
       </c>
     </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>170</v>
       </c>
@@ -9736,7 +9740,7 @@
         <v>-1.26287479999999E-2</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>171</v>
       </c>
@@ -9786,7 +9790,7 @@
         <v>-3.3567386399999899E-2</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>172</v>
       </c>
@@ -9836,7 +9840,7 @@
         <v>-4.6810740000000099E-3</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>173</v>
       </c>
@@ -9886,7 +9890,7 @@
         <v>-1.9720387199999901E-2</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>174</v>
       </c>
@@ -9936,7 +9940,7 @@
         <v>-5.4865559999999801E-3</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>175</v>
       </c>
@@ -9986,7 +9990,7 @@
         <v>-1.8925436399999902E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>176</v>
       </c>
@@ -10036,7 +10040,7 @@
         <v>-1.4608562E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>177</v>
       </c>
@@ -10086,7 +10090,7 @@
         <v>-1.94127999999999E-2</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>178</v>
       </c>
@@ -10136,7 +10140,7 @@
         <v>2.84140404E-2</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>179</v>
       </c>
@@ -10186,7 +10190,7 @@
         <v>-2.8621938399999901E-2</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>180</v>
       </c>
@@ -10236,7 +10240,7 @@
         <v>-2.3967914399999998E-2</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>181</v>
       </c>
@@ -10286,7 +10290,7 @@
         <v>1.730826E-3</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>182</v>
       </c>
@@ -10336,7 +10340,7 @@
         <v>3.9104748000000104E-3</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>183</v>
       </c>
@@ -10386,7 +10390,7 @@
         <v>-5.2340896000000097E-3</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>184</v>
       </c>
@@ -10436,7 +10440,7 @@
         <v>3.0001127999999998E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>185</v>
       </c>
@@ -10486,7 +10490,7 @@
         <v>2.4770592399999999E-2</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>186</v>
       </c>
@@ -10536,7 +10540,7 @@
         <v>3.2322125999999902E-2</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>187</v>
       </c>
@@ -10586,7 +10590,7 @@
         <v>-7.6230073076922998E-3</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>188</v>
       </c>
@@ -10636,7 +10640,7 @@
         <v>-6.2729380769230699E-3</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>189</v>
       </c>
@@ -10686,7 +10690,7 @@
         <v>-1.4072707307692301E-2</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>190</v>
       </c>
@@ -10736,7 +10740,7 @@
         <v>-4.2897074230769203E-2</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>191</v>
       </c>
@@ -10786,7 +10790,7 @@
         <v>-6.9921458076923002E-2</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>192</v>
       </c>
@@ -10836,7 +10840,7 @@
         <v>-3.9312069999999998E-2</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>193</v>
       </c>
@@ -10886,7 +10890,7 @@
         <v>-1.3176145E-2</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>194</v>
       </c>
@@ -10936,7 +10940,7 @@
         <v>-2.3181711538461498E-2</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>195</v>
       </c>
@@ -10986,7 +10990,7 @@
         <v>-1.22626192307692E-2</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A197">
         <v>196</v>
       </c>
@@ -11036,7 +11040,7 @@
         <v>2.0717103076923E-2</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>197</v>
       </c>
@@ -11086,7 +11090,7 @@
         <v>1.91043515384615E-2</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>198</v>
       </c>
@@ -11136,7 +11140,7 @@
         <v>1.13936911538461E-2</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>199</v>
       </c>
@@ -11186,7 +11190,7 @@
         <v>8.0700549999999996E-3</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>200</v>
       </c>
@@ -11236,7 +11240,7 @@
         <v>1.2661719230769201E-2</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A202">
         <v>201</v>
       </c>
@@ -11286,7 +11290,7 @@
         <v>1.1750454230769199E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A203">
         <v>202</v>
       </c>
@@ -11336,7 +11340,7 @@
         <v>-4.3588230769230699E-3</v>
       </c>
     </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A204">
         <v>203</v>
       </c>
@@ -11386,7 +11390,7 @@
         <v>-4.3079999999999798E-5</v>
       </c>
     </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A205">
         <v>204</v>
       </c>
@@ -11436,7 +11440,7 @@
         <v>3.1083707692307698E-3</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A206">
         <v>205</v>
       </c>
@@ -11486,7 +11490,7 @@
         <v>-4.8501949230769198E-2</v>
       </c>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A207">
         <v>206</v>
       </c>
@@ -11536,7 +11540,7 @@
         <v>-3.5612535769230701E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A208">
         <v>207</v>
       </c>
@@ -11586,7 +11590,7 @@
         <v>-3.7370544230769201E-2</v>
       </c>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A209">
         <v>208</v>
       </c>
@@ -11636,7 +11640,7 @@
         <v>-4.8398943076923003E-2</v>
       </c>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A210">
         <v>209</v>
       </c>
@@ -11686,7 +11690,7 @@
         <v>-4.5124831538461502E-2</v>
       </c>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A211">
         <v>210</v>
       </c>
@@ -11736,7 +11740,7 @@
         <v>-4.0824941538461501E-2</v>
       </c>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A212">
         <v>211</v>
       </c>
@@ -11786,7 +11790,7 @@
         <v>-2.6929980769230702E-3</v>
       </c>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A213">
         <v>212</v>
       </c>
@@ -11836,7 +11840,7 @@
         <v>-2.50341384615384E-3</v>
       </c>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A214">
         <v>213</v>
       </c>
@@ -11886,7 +11890,7 @@
         <v>1.25482326923076E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A215">
         <v>214</v>
       </c>
@@ -11936,7 +11940,7 @@
         <v>5.11670692307692E-3</v>
       </c>
     </row>
-    <row r="216" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A216">
         <v>215</v>
       </c>
@@ -11986,7 +11990,7 @@
         <v>-2.6833630769230702E-3</v>
       </c>
     </row>
-    <row r="217" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A217">
         <v>216</v>
       </c>
@@ -12036,7 +12040,7 @@
         <v>1.6459523076922999E-2</v>
       </c>
     </row>
-    <row r="218" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A218">
         <v>217</v>
       </c>
@@ -12086,7 +12090,7 @@
         <v>8.0449149999999997E-3</v>
       </c>
     </row>
-    <row r="219" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A219">
         <v>218</v>
       </c>
@@ -12136,7 +12140,7 @@
         <v>3.9555972307692297E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A220">
         <v>219</v>
       </c>
@@ -12186,7 +12190,7 @@
         <v>4.39240115384615E-3</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A221">
         <v>220</v>
       </c>
@@ -12236,7 +12240,7 @@
         <v>8.3788007692307698E-3</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A222">
         <v>221</v>
       </c>
@@ -12286,7 +12290,7 @@
         <v>3.8143673076923E-3</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A223">
         <v>222</v>
       </c>
@@ -12336,7 +12340,7 @@
         <v>4.98469961538461E-3</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A224">
         <v>223</v>
       </c>
@@ -12386,7 +12390,7 @@
         <v>-9.7843719230769205E-3</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A225">
         <v>224</v>
       </c>
@@ -12436,7 +12440,7 @@
         <v>-8.8409873076923003E-3</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A226">
         <v>225</v>
       </c>
@@ -12486,7 +12490,7 @@
         <v>-2.3986223076923E-3</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A227">
         <v>226</v>
       </c>
@@ -12536,7 +12540,7 @@
         <v>-1.37151361538461E-2</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A228">
         <v>227</v>
       </c>
@@ -12586,7 +12590,7 @@
         <v>-1.40864126923076E-2</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A229">
         <v>228</v>
       </c>
@@ -12636,7 +12640,7 @@
         <v>-1.6277986538461499E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A230">
         <v>229</v>
       </c>
@@ -12686,7 +12690,7 @@
         <v>2.9859796153846102E-3</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A231">
         <v>230</v>
       </c>
@@ -12736,7 +12740,7 @@
         <v>1.03480007692307E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A232">
         <v>231</v>
       </c>
@@ -12786,7 +12790,7 @@
         <v>3.2499299999999998E-3</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A233">
         <v>232</v>
       </c>
@@ -12836,7 +12840,7 @@
         <v>-1.41347949999999E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A234">
         <v>233</v>
       </c>
@@ -12886,7 +12890,7 @@
         <v>4.0543503846153803E-3</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A235">
         <v>234</v>
       </c>
@@ -12936,7 +12940,7 @@
         <v>-2.0006690384615299E-2</v>
       </c>
     </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A236">
         <v>235</v>
       </c>
@@ -12986,7 +12990,7 @@
         <v>-2.8493367692307599E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A237">
         <v>236</v>
       </c>
@@ -13036,7 +13040,7 @@
         <v>-2.1408105E-2</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A238">
         <v>237</v>
       </c>
@@ -13086,7 +13090,7 @@
         <v>-1.6278972692307599E-2</v>
       </c>
     </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A239">
         <v>238</v>
       </c>
@@ -13136,7 +13140,7 @@
         <v>6.7474269230769204E-3</v>
       </c>
     </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A240">
         <v>239</v>
       </c>
@@ -13186,7 +13190,7 @@
         <v>3.5250653846153598E-4</v>
       </c>
     </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A241">
         <v>240</v>
       </c>
@@ -13236,7 +13240,7 @@
         <v>5.4015596153846098E-3</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A242">
         <v>241</v>
       </c>
@@ -13286,7 +13290,7 @@
         <v>-4.6332873076923003E-3</v>
       </c>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A243">
         <v>242</v>
       </c>
@@ -13336,7 +13340,7 @@
         <v>-1.5609390769230701E-2</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A244">
         <v>243</v>
       </c>
@@ -13386,7 +13390,7 @@
         <v>4.4776953846153798E-3</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A245">
         <v>244</v>
       </c>
@@ -13436,7 +13440,7 @@
         <v>-1.3367978846153801E-2</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A246">
         <v>245</v>
       </c>
@@ -13486,7 +13490,7 @@
         <v>-5.0521075384615297E-2</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A247">
         <v>246</v>
       </c>
@@ -13536,7 +13540,7 @@
         <v>-1.31982238461538E-2</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A248">
         <v>247</v>
       </c>
@@ -13586,7 +13590,7 @@
         <v>2.2335833461538401E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A249">
         <v>248</v>
       </c>
@@ -13636,7 +13640,7 @@
         <v>-1.8319408846153799E-2</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A250">
         <v>249</v>
       </c>
@@ -13686,7 +13690,7 @@
         <v>1.7372911538461499E-2</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A251">
         <v>250</v>
       </c>
@@ -13736,7 +13740,7 @@
         <v>2.3170753846153799E-3</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A252">
         <v>251</v>
       </c>
@@ -13786,7 +13790,7 @@
         <v>-9.3619846153846105E-4</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A253">
         <v>252</v>
       </c>
@@ -13836,7 +13840,7 @@
         <v>-6.5218526923076902E-3</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A254">
         <v>253</v>
       </c>
@@ -13886,7 +13890,7 @@
         <v>-1.0478491538461501E-2</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A255">
         <v>254</v>
       </c>
@@ -13936,7 +13940,7 @@
         <v>-1.7200073076922999E-2</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A256">
         <v>255</v>
       </c>
@@ -13986,7 +13990,7 @@
         <v>-1.6506783076923E-2</v>
       </c>
     </row>
-    <row r="257" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A257">
         <v>256</v>
       </c>
@@ -14036,7 +14040,7 @@
         <v>2.3993699999999901E-3</v>
       </c>
     </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A258">
         <v>257</v>
       </c>
@@ -14086,7 +14090,7 @@
         <v>-2.4490703846153801E-3</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A259">
         <v>258</v>
       </c>
@@ -14136,7 +14140,7 @@
         <v>7.0207573076923003E-3</v>
       </c>
     </row>
-    <row r="260" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A260">
         <v>259</v>
       </c>
@@ -14186,7 +14190,7 @@
         <v>1.31359234615384E-2</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A261">
         <v>260</v>
       </c>
@@ -14236,7 +14240,7 @@
         <v>9.9447219230769206E-3</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A262">
         <v>261</v>
       </c>
@@ -14286,7 +14290,7 @@
         <v>-1.6571410000000002E-2</v>
       </c>
     </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A263">
         <v>262</v>
       </c>
@@ -14336,7 +14340,7 @@
         <v>2.73534415384615E-2</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A264">
         <v>263</v>
       </c>
@@ -14386,7 +14390,7 @@
         <v>-5.2150546153846098E-3</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A265">
         <v>264</v>
       </c>
@@ -14436,7 +14440,7 @@
         <v>7.5477092307692298E-3</v>
       </c>
     </row>
-    <row r="266" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A266">
         <v>265</v>
       </c>
@@ -14486,7 +14490,7 @@
         <v>1.3326799230769199E-2</v>
       </c>
     </row>
-    <row r="267" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A267">
         <v>266</v>
       </c>
@@ -14536,7 +14540,7 @@
         <v>1.88403923076923E-2</v>
       </c>
     </row>
-    <row r="268" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A268">
         <v>267</v>
       </c>
@@ -14586,7 +14590,7 @@
         <v>1.5669708461538399E-2</v>
       </c>
     </row>
-    <row r="269" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A269">
         <v>268</v>
       </c>
@@ -14636,7 +14640,7 @@
         <v>8.0336534615384602E-3</v>
       </c>
     </row>
-    <row r="270" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A270">
         <v>269</v>
       </c>
@@ -14686,7 +14690,7 @@
         <v>5.7111273076923003E-3</v>
       </c>
     </row>
-    <row r="271" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A271">
         <v>270</v>
       </c>
@@ -14736,7 +14740,7 @@
         <v>5.3918038461538002E-4</v>
       </c>
     </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A272">
         <v>271</v>
       </c>
@@ -14786,7 +14790,7 @@
         <v>4.1960005000000002E-2</v>
       </c>
     </row>
-    <row r="273" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A273">
         <v>272</v>
       </c>
@@ -14836,7 +14840,7 @@
         <v>-1.3429776923076901E-3</v>
       </c>
     </row>
-    <row r="274" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A274">
         <v>273</v>
       </c>
@@ -14886,7 +14890,7 @@
         <v>2.34218988461538E-2</v>
       </c>
     </row>
-    <row r="275" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A275">
         <v>274</v>
       </c>
@@ -14936,7 +14940,7 @@
         <v>7.5053023076922997E-3</v>
       </c>
     </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A276">
         <v>275</v>
       </c>
@@ -14986,7 +14990,7 @@
         <v>1.9351290384615302E-2</v>
       </c>
     </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A277">
         <v>276</v>
       </c>
@@ -15036,7 +15040,7 @@
         <v>9.2099711538461502E-3</v>
       </c>
     </row>
-    <row r="278" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A278">
         <v>277</v>
       </c>
@@ -15086,7 +15090,7 @@
         <v>3.7831023076923E-3</v>
       </c>
     </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A279">
         <v>278</v>
       </c>
@@ -15136,7 +15140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A280">
         <v>279</v>
       </c>
@@ -15186,7 +15190,7 @@
         <v>2.6809707692307598E-3</v>
       </c>
     </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A281">
         <v>280</v>
       </c>
@@ -15236,7 +15240,7 @@
         <v>5.7017319230769203E-3</v>
       </c>
     </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A282">
         <v>281</v>
       </c>
@@ -15286,7 +15290,7 @@
         <v>8.0103911538461497E-3</v>
       </c>
     </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A283">
         <v>282</v>
       </c>
@@ -15336,7 +15340,7 @@
         <v>1.8776105000000001E-2</v>
       </c>
     </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A284">
         <v>283</v>
       </c>
@@ -15386,7 +15390,7 @@
         <v>2.1457027307692299E-2</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A285">
         <v>284</v>
       </c>
@@ -15436,7 +15440,7 @@
         <v>-1.65589692307692E-3</v>
       </c>
     </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A286">
         <v>285</v>
       </c>
@@ -15486,7 +15490,7 @@
         <v>1.11177215384615E-2</v>
       </c>
     </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A287">
         <v>286</v>
       </c>
@@ -15536,7 +15540,7 @@
         <v>-3.4682111538461499E-2</v>
       </c>
     </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A288">
         <v>287</v>
       </c>
@@ -15586,7 +15590,7 @@
         <v>-2.9569223076922999E-3</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A289">
         <v>288</v>
       </c>
@@ -15636,7 +15640,7 @@
         <v>-3.2875905384615302E-2</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A290">
         <v>289</v>
       </c>
@@ -15686,7 +15690,7 @@
         <v>6.4894034615384597E-3</v>
       </c>
     </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A291">
         <v>290</v>
       </c>
@@ -15736,7 +15740,7 @@
         <v>2.6315009999999899E-2</v>
       </c>
     </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A292">
         <v>291</v>
       </c>
@@ -15786,7 +15790,7 @@
         <v>2.0220283846153798E-2</v>
       </c>
     </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A293">
         <v>292</v>
       </c>
@@ -15836,7 +15840,7 @@
         <v>-3.4561296153846101E-3</v>
       </c>
     </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A294">
         <v>293</v>
       </c>
@@ -15886,7 +15890,7 @@
         <v>-9.1049991153846099E-2</v>
       </c>
     </row>
-    <row r="295" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A295">
         <v>294</v>
       </c>
@@ -15936,7 +15940,7 @@
         <v>4.6862226923076898E-3</v>
       </c>
     </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A296">
         <v>295</v>
       </c>
@@ -15986,7 +15990,7 @@
         <v>4.2441561153846098E-2</v>
       </c>
     </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A297">
         <v>296</v>
       </c>
@@ -16036,7 +16040,7 @@
         <v>2.4533079999999999E-2</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A298">
         <v>297</v>
       </c>
@@ -16086,7 +16090,7 @@
         <v>1.72068826923076E-2</v>
       </c>
     </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A299">
         <v>298</v>
       </c>
@@ -16136,7 +16140,7 @@
         <v>-8.9519230769230709E-3</v>
       </c>
     </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A300">
         <v>299</v>
       </c>
@@ -16186,7 +16190,7 @@
         <v>-1.2558869615384599E-2</v>
       </c>
     </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A301">
         <v>300</v>
       </c>
@@ -16236,7 +16240,7 @@
         <v>-8.0018911538461499E-3</v>
       </c>
     </row>
-    <row r="302" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A302">
         <v>301</v>
       </c>
@@ -16286,7 +16290,7 @@
         <v>3.5699876923076901E-3</v>
       </c>
     </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A303">
         <v>302</v>
       </c>
@@ -16336,7 +16340,7 @@
         <v>1.9809396153846102E-3</v>
       </c>
     </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A304">
         <v>303</v>
       </c>
@@ -16386,7 +16390,7 @@
         <v>6.5392384615384496E-4</v>
       </c>
     </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A305">
         <v>304</v>
       </c>
@@ -16436,7 +16440,7 @@
         <v>-8.0693815384615293E-3</v>
       </c>
     </row>
-    <row r="306" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A306">
         <v>305</v>
       </c>
@@ -16486,7 +16490,7 @@
         <v>-8.1787065384615401E-3</v>
       </c>
     </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A307">
         <v>306</v>
       </c>
@@ -16536,7 +16540,7 @@
         <v>-1.0188736153846099E-2</v>
       </c>
     </row>
-    <row r="308" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A308">
         <v>307</v>
       </c>
@@ -16586,7 +16590,7 @@
         <v>-2.3840926923076899E-3</v>
       </c>
     </row>
-    <row r="309" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A309">
         <v>308</v>
       </c>
@@ -16636,7 +16640,7 @@
         <v>1.04728E-3</v>
       </c>
     </row>
-    <row r="310" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A310">
         <v>309</v>
       </c>
@@ -16686,7 +16690,7 @@
         <v>1.4631703846153801E-3</v>
       </c>
     </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A311">
         <v>310</v>
       </c>
@@ -16736,7 +16740,7 @@
         <v>2.4627050000000001E-2</v>
       </c>
     </row>
-    <row r="312" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A312">
         <v>311</v>
       </c>
@@ -16786,7 +16790,7 @@
         <v>5.3395036153846102E-2</v>
       </c>
     </row>
-    <row r="313" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A313">
         <v>312</v>
       </c>
@@ -16836,7 +16840,7 @@
         <v>1.1586331538461499E-2</v>
       </c>
     </row>
-    <row r="314" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A314">
         <v>313</v>
       </c>
@@ -16886,7 +16890,7 @@
         <v>8.2934569230769199E-3</v>
       </c>
     </row>
-    <row r="315" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A315">
         <v>314</v>
       </c>
@@ -16936,7 +16940,7 @@
         <v>4.3207307692307703E-5</v>
       </c>
     </row>
-    <row r="316" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A316">
         <v>315</v>
       </c>
@@ -16986,7 +16990,7 @@
         <v>1.1024047307692301E-2</v>
       </c>
     </row>
-    <row r="317" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A317">
         <v>316</v>
       </c>
@@ -17036,7 +17040,7 @@
         <v>-3.7282509230769201E-2</v>
       </c>
     </row>
-    <row r="318" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A318">
         <v>317</v>
       </c>
@@ -17086,7 +17090,7 @@
         <v>-3.7088817307692298E-2</v>
       </c>
     </row>
-    <row r="319" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A319">
         <v>318</v>
       </c>
@@ -17136,7 +17140,7 @@
         <v>-2.0481454615384601E-2</v>
       </c>
     </row>
-    <row r="320" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A320">
         <v>319</v>
       </c>
@@ -17186,7 +17190,7 @@
         <v>4.1549138461538402E-3</v>
       </c>
     </row>
-    <row r="321" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A321">
         <v>320</v>
       </c>
@@ -17236,7 +17240,7 @@
         <v>1.3870396153846101E-3</v>
       </c>
     </row>
-    <row r="322" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A322">
         <v>321</v>
       </c>
@@ -17286,7 +17290,7 @@
         <v>2.61192169230769E-2</v>
       </c>
     </row>
-    <row r="323" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A323">
         <v>322</v>
       </c>
@@ -17336,7 +17340,7 @@
         <v>1.12009153846153E-2</v>
       </c>
     </row>
-    <row r="324" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A324">
         <v>323</v>
       </c>
@@ -17386,7 +17390,7 @@
         <v>-7.1741730769230702E-3</v>
       </c>
     </row>
-    <row r="325" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A325">
         <v>324</v>
       </c>
@@ -17436,7 +17440,7 @@
         <v>4.8842215384615299E-3</v>
       </c>
     </row>
-    <row r="327" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>16</v>
       </c>
@@ -17501,7 +17505,7 @@
         <v>-5.5541811881460179E-3</v>
       </c>
     </row>
-    <row r="328" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A328" s="14" t="s">
         <v>17</v>
       </c>
@@ -17566,7 +17570,7 @@
         <v>-3.1527420426065199E-3</v>
       </c>
     </row>
-    <row r="329" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>18</v>
       </c>
@@ -17631,7 +17635,7 @@
         <v>-0.21105627333333299</v>
       </c>
     </row>
-    <row r="330" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>19</v>
       </c>
@@ -17696,7 +17700,7 @@
         <v>0.106106966666666</v>
       </c>
     </row>
-    <row r="332" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>20</v>
       </c>
@@ -17761,7 +17765,7 @@
         <v>-1.8160065094017058E-2</v>
       </c>
     </row>
-    <row r="333" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>21</v>
       </c>
@@ -17826,7 +17830,7 @@
         <v>-6.7086922433862361E-3</v>
       </c>
     </row>
-    <row r="334" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>22</v>
       </c>
@@ -17891,7 +17895,7 @@
         <v>5.0184561538460797E-4</v>
       </c>
     </row>
-    <row r="335" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>23</v>
       </c>
@@ -17956,7 +17960,7 @@
         <v>9.3205487529137588E-3</v>
       </c>
     </row>
-    <row r="336" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>27</v>
       </c>
@@ -18021,7 +18025,7 @@
         <v>2.7480613846930818E-2</v>
       </c>
     </row>
-    <row r="337" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A337" s="11" t="s">
         <v>34</v>
       </c>
@@ -18086,7 +18090,7 @@
         <v>4.5801023078218027E-3</v>
       </c>
     </row>
-    <row r="339" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
         <v>15</v>
       </c>
@@ -18136,7 +18140,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="340" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
         <v>24</v>
       </c>
@@ -18201,7 +18205,7 @@
         <v>-9.0000000000000011E-3</v>
       </c>
     </row>
-    <row r="341" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
         <v>25</v>
       </c>
@@ -18266,7 +18270,7 @@
         <v>-3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="342" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A342" s="3" t="s">
         <v>35</v>
       </c>
@@ -18316,7 +18320,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="343" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
         <v>26</v>
       </c>
@@ -18390,12 +18394,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA9E5EE3-BE15-40A4-B60C-E3A8AEA81B11}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="43.109375" customWidth="1"/>
+    <col min="1" max="1" width="43.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="16" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="16" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
         <v>36</v>
       </c>
@@ -18412,7 +18416,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -18429,7 +18433,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -18446,29 +18450,29 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>54</v>
       </c>
       <c r="B4">
-        <v>-0.05</v>
+        <v>-0.04</v>
       </c>
       <c r="C4">
-        <v>-0.02</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="D4">
-        <v>0.02</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E4">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>51</v>
       </c>
       <c r="B5">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.04</v>
       </c>
       <c r="C5">
         <v>-1.4999999999999999E-2</v>
@@ -18477,49 +18481,49 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="E5">
-        <v>2.5000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>52</v>
       </c>
       <c r="B6">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.04</v>
       </c>
       <c r="C6">
-        <v>-0.01</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="D6">
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E6">
-        <v>2.5000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>53</v>
       </c>
       <c r="B7">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.04</v>
       </c>
       <c r="C7">
-        <v>-0.01</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="D7">
-        <v>0.01</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E7">
-        <v>2.5000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>38</v>
       </c>
       <c r="B8">
-        <v>-0.4</v>
+        <v>-0.3</v>
       </c>
       <c r="C8">
         <v>-0.1</v>
@@ -18528,15 +18532,15 @@
         <v>0.1</v>
       </c>
       <c r="E8">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>48</v>
       </c>
       <c r="B9">
-        <v>-0.5</v>
+        <v>-0.75</v>
       </c>
       <c r="C9">
         <v>-0.3</v>
@@ -18545,66 +18549,66 @@
         <v>0.3</v>
       </c>
       <c r="E9">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>39</v>
       </c>
       <c r="B10">
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="C10">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="D10">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="E10">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>40</v>
       </c>
       <c r="B11">
-        <v>-0.3</v>
+        <v>-0.4</v>
       </c>
       <c r="C11">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="D11">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="E11">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>41</v>
       </c>
       <c r="B12">
-        <v>-0.25</v>
+        <v>-0.35</v>
       </c>
       <c r="C12">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="D12">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="E12">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>49</v>
       </c>
       <c r="B13">
-        <v>-0.5</v>
+        <v>-0.8</v>
       </c>
       <c r="C13">
         <v>-0.3</v>
@@ -18613,10 +18617,10 @@
         <v>0.3</v>
       </c>
       <c r="E13">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>42</v>
       </c>
@@ -18624,16 +18628,16 @@
         <v>-0.5</v>
       </c>
       <c r="C14">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="D14">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E14">
         <v>0.5</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -18641,16 +18645,16 @@
         <v>-30</v>
       </c>
       <c r="C15">
-        <v>-15</v>
+        <v>-10</v>
       </c>
       <c r="D15">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E15">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -18667,24 +18671,24 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>45</v>
       </c>
       <c r="B17">
+        <v>-30</v>
+      </c>
+      <c r="C17">
         <v>-10</v>
       </c>
-      <c r="C17">
-        <v>-5</v>
-      </c>
       <c r="D17">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E17">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -18701,7 +18705,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -18718,7 +18722,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Namen Anpassungen und Farben Temperatur reverse in delta
</commit_message>
<xml_diff>
--- a/appdata/threshold_definitions_delta_de.xlsx
+++ b/appdata/threshold_definitions_delta_de.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zhaw-my.sharepoint.com/personal/hedd_zhaw_ch/Documents/Dashboard Squarefoot Projekt/Squarefoot/Squarefoot code/squarefoot/appdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:9_{36C0AF89-E858-44E3-B955-074CA1A8DB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1355B14B-7469-457B-9C2A-CD7D9FC758C6}"/>
+  <xr:revisionPtr revIDLastSave="179" documentId="13_ncr:9_{36C0AF89-E858-44E3-B955-074CA1A8DB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D2D7555-E682-4433-9087-601DD503A0C5}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="1770" windowWidth="21600" windowHeight="11295" xr2:uid="{DF7BF7E8-8078-438A-9C9E-DC555A1DD317}"/>
+    <workbookView xWindow="4395" yWindow="2715" windowWidth="21600" windowHeight="11295" xr2:uid="{DF7BF7E8-8078-438A-9C9E-DC555A1DD317}"/>
   </bookViews>
   <sheets>
     <sheet name="Schwellenwerte" sheetId="3" r:id="rId1"/>
@@ -44,15 +44,6 @@
     <t>anzahl_arten</t>
   </si>
   <si>
-    <t>temperatur</t>
-  </si>
-  <si>
-    <t>reaktion</t>
-  </si>
-  <si>
-    <t>feuchtigkeit</t>
-  </si>
-  <si>
     <t>licht</t>
   </si>
   <si>
@@ -74,9 +65,6 @@
     <t>konkurrenzstrategie</t>
   </si>
   <si>
-    <t>na0ehrstoff</t>
-  </si>
-  <si>
     <t>mahdvertra0eglichkeit</t>
   </si>
   <si>
@@ -105,6 +93,18 @@
   </si>
   <si>
     <t>starke Abnahme</t>
+  </si>
+  <si>
+    <t>temperaturzahl</t>
+  </si>
+  <si>
+    <t>na0ehrstoffzahl</t>
+  </si>
+  <si>
+    <t>reaktionszahl</t>
+  </si>
+  <si>
+    <t>feuchtigkeitszahl</t>
   </si>
 </sst>
 </file>
@@ -637,10 +637,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -971,16 +967,16 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1002,7 +998,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>0.15</v>
@@ -1019,7 +1015,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B4">
         <v>0.04</v>
@@ -1036,7 +1032,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>0.04</v>
@@ -1053,7 +1049,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>0.04</v>
@@ -1070,7 +1066,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <v>0.04</v>
@@ -1087,7 +1083,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>0.3</v>
@@ -1104,7 +1100,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>0.75</v>
@@ -1121,7 +1117,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>0.6</v>
@@ -1138,7 +1134,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>0.4</v>
@@ -1155,7 +1151,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>0.35</v>
@@ -1172,7 +1168,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B13">
         <v>0.8</v>
@@ -1189,7 +1185,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>0.5</v>
@@ -1206,7 +1202,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B15">
         <v>30</v>
@@ -1223,7 +1219,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B16">
         <v>30</v>
@@ -1240,7 +1236,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B17">
         <v>30</v>
@@ -1274,7 +1270,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B19">
         <v>0.1</v>
@@ -1291,7 +1287,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>0.1</v>

</xml_diff>